<commit_message>
Add auth/login, Postgres+Drizzle backend, and settings/theme UI (WIP demo)
Isolated on this branch so Vercel builds it as a separate preview
deployment, independent of production.
</commit_message>
<xml_diff>
--- a/app/TOPUP_TEMPLATE_V1.xlsx
+++ b/app/TOPUP_TEMPLATE_V1.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejboy\Desktop\dashbaord_project\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02ED42DD-B8BF-40AC-9B4E-A2075106BEA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B1D5D8-8F74-4623-9ECD-50046A38DE25}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{11DBCEFB-88F7-48A5-B32D-B2D8ED80C28F}"/>
   </bookViews>
   <sheets>
     <sheet name="TopUp" sheetId="1" r:id="rId1"/>
+    <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Brand</t>
   </si>
@@ -43,6 +44,15 @@
   </si>
   <si>
     <t>Agent</t>
+  </si>
+  <si>
+    <t>Bundle Transfer In</t>
+  </si>
+  <si>
+    <t>Internal Transfer In</t>
+  </si>
+  <si>
+    <t>Top Up</t>
   </si>
 </sst>
 </file>
@@ -496,5 +506,45 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{54B643A9-C9C4-405A-A572-14992A014F9D}">
+          <x14:formula1>
+            <xm:f>Notes!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>F3:F250</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43D5CDAA-063C-4885-B453-6C69C384A310}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>